<commit_message>
amended business cost table 8a
</commit_message>
<xml_diff>
--- a/data/balance.xlsx
+++ b/data/balance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11113"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livelancsac-my.sharepoint.com/personal/daryanto_lancaster_ac_uk/Documents/numbook/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahmaddaryanto/Documents/GitHub/numbook/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{10964F35-A639-E147-A62A-E63F27CF6A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD4635C5-EF85-EC42-87DA-3775CF422B20}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB1C8BCD-8AA8-2248-A402-405EBF1A82AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1860" windowWidth="28040" windowHeight="17440" xr2:uid="{BA12D64F-0178-424C-87DA-7EEDD185031D}"/>
+    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="15760" xr2:uid="{BA12D64F-0178-424C-87DA-7EEDD185031D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Variable costs per job</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Cost (£)</t>
+  </si>
+  <si>
+    <t>Your Business (December)</t>
   </si>
 </sst>
 </file>
@@ -85,12 +88,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -105,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -114,7 +123,10 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -132,10 +144,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -445,7 +453,9 @@
   <sheetData>
     <row r="2" spans="1:8" ht="26" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -534,10 +544,10 @@
     </row>
     <row r="9" spans="1:8" ht="26" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="5">
         <v>50</v>
       </c>
       <c r="D9" s="1"/>

</xml_diff>